<commit_message>
Launch CSBT Exchange and fix production build
</commit_message>
<xml_diff>
--- a/source-data/trading-data.pre-elve-sync.backup.xlsx
+++ b/source-data/trading-data.pre-elve-sync.backup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="26400" windowHeight="10830" activeTab="10"/>
+    <workbookView windowWidth="26400" windowHeight="10830" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -28743,7 +28743,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D14 A15:B15 D15 A16:D25 A26:B26 D26 A27:D1000" numberStoredAsText="1"/>
+    <ignoredError sqref="A27:D1000 D26 A26:B26 A16:D25 D15 A15:B15 A1:D14" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -61830,7 +61830,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I1770" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:B1 D1:I1 A2:I1770" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Refresh Elve values and regenerate trading data
</commit_message>
<xml_diff>
--- a/source-data/trading-data.pre-elve-sync.backup.xlsx
+++ b/source-data/trading-data.pre-elve-sync.backup.xlsx
@@ -5202,7 +5202,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1007"/>
+  <dimension ref="A1:I1009"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="24.4416666666667"/>
     <col min="2" max="2" customWidth="1" width="49"/>
@@ -5376,10 +5376,10 @@
         <v>7</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H6">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I6" t="str">
         <v>2D Doggy</v>
@@ -5495,7 +5495,7 @@
         <v>530</v>
       </c>
       <c r="H10">
-        <v>1925</v>
+        <v>1930</v>
       </c>
       <c r="I10" t="str">
         <v>African Wild Dog</v>
@@ -5692,13 +5692,13 @@
         <v>2520</v>
       </c>
       <c r="F17">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G17">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H17">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="I17" t="str">
         <v>Alpaca</v>
@@ -6243,13 +6243,13 @@
         <v>330</v>
       </c>
       <c r="F36">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="G36">
-        <v>6.79</v>
+        <v>6.86</v>
       </c>
       <c r="H36">
-        <v>27.5</v>
+        <v>27.8</v>
       </c>
       <c r="I36" t="str">
         <v>Astronaut Gorilla</v>
@@ -6475,13 +6475,13 @@
         <v>1800</v>
       </c>
       <c r="F44">
-        <v>9.5</v>
+        <v>10.75</v>
       </c>
       <c r="G44">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="H44">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="I44" t="str">
         <v>Bald Eagle</v>
@@ -6536,10 +6536,10 @@
         <v>167</v>
       </c>
       <c r="G46">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="H46">
-        <v>1980</v>
+        <v>2000</v>
       </c>
       <c r="I46" t="str">
         <v>Balloon Unicorn</v>
@@ -6684,7 +6684,7 @@
         <v>2170</v>
       </c>
       <c r="H51">
-        <v>6950</v>
+        <v>7000</v>
       </c>
       <c r="I51" t="str">
         <v>Bat Dragon</v>
@@ -7374,13 +7374,13 @@
         <v>24120</v>
       </c>
       <c r="F75">
-        <v>148</v>
+        <v>148.5</v>
       </c>
       <c r="G75">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="H75">
-        <v>2050</v>
+        <v>2100</v>
       </c>
       <c r="I75" t="str">
         <v>Blazing Lion</v>
@@ -7983,13 +7983,13 @@
         <v>110</v>
       </c>
       <c r="F96">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="G96">
-        <v>2.35</v>
+        <v>2.45</v>
       </c>
       <c r="H96">
-        <v>10.25</v>
+        <v>10.75</v>
       </c>
       <c r="I96" t="str">
         <v>Burning Bunny</v>
@@ -8012,13 +8012,13 @@
         <v>3090</v>
       </c>
       <c r="F97">
-        <v>18.75</v>
+        <v>19.75</v>
       </c>
       <c r="G97">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="H97">
-        <v>270</v>
+        <v>290</v>
       </c>
       <c r="I97" t="str">
         <v>Bush Elephant</v>
@@ -8041,13 +8041,13 @@
         <v>190</v>
       </c>
       <c r="F98">
-        <v>0.67</v>
+        <v>0.69</v>
       </c>
       <c r="G98">
-        <v>4.15</v>
+        <v>4.25</v>
       </c>
       <c r="H98">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="I98" t="str">
         <v>Business Monkey</v>
@@ -8070,13 +8070,13 @@
         <v>2640</v>
       </c>
       <c r="F99">
-        <v>26.25</v>
+        <v>26.5</v>
       </c>
       <c r="G99">
         <v>58</v>
       </c>
       <c r="H99">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="I99" t="str">
         <v>Cabbit</v>
@@ -8273,13 +8273,13 @@
         <v>100</v>
       </c>
       <c r="F106">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="G106">
-        <v>2.15</v>
+        <v>2.3</v>
       </c>
       <c r="H106">
-        <v>9.25</v>
+        <v>10</v>
       </c>
       <c r="I106" t="str">
         <v>Candy Cane Snail</v>
@@ -8670,13 +8670,13 @@
         <v>260</v>
       </c>
       <c r="F120">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="G120">
-        <v>5.9</v>
+        <v>5.95</v>
       </c>
       <c r="H120">
-        <v>24.6</v>
+        <v>24.8</v>
       </c>
       <c r="I120" t="str">
         <v>Chef Gorilla</v>
@@ -9691,7 +9691,7 @@
         <v>397</v>
       </c>
       <c r="H155">
-        <v>1275</v>
+        <v>1210</v>
       </c>
       <c r="I155" t="str">
         <v>Crow</v>
@@ -9714,13 +9714,13 @@
         <v>14040</v>
       </c>
       <c r="F156">
-        <v>134</v>
+        <v>134.5</v>
       </c>
       <c r="G156">
-        <v>320</v>
+        <v>338</v>
       </c>
       <c r="H156">
-        <v>1250</v>
+        <v>1350</v>
       </c>
       <c r="I156" t="str">
         <v>Cryptid</v>
@@ -9830,7 +9830,7 @@
         <v>9420</v>
       </c>
       <c r="F160">
-        <v>58.75</v>
+        <v>59</v>
       </c>
       <c r="G160">
         <v>198</v>
@@ -11132,13 +11132,13 @@
         <v>2000</v>
       </c>
       <c r="F205">
-        <v>15</v>
+        <v>16.25</v>
       </c>
       <c r="G205">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H205">
-        <v>254</v>
+        <v>270</v>
       </c>
       <c r="I205" t="str">
         <v>Emperor Gorilla</v>
@@ -11399,7 +11399,7 @@
         <v>200</v>
       </c>
       <c r="H214">
-        <v>730</v>
+        <v>715</v>
       </c>
       <c r="I214" t="str">
         <v>Evil Unicorn</v>
@@ -11422,10 +11422,10 @@
         <v>2000</v>
       </c>
       <c r="F215">
-        <v>15.75</v>
+        <v>16.5</v>
       </c>
       <c r="G215">
-        <v>44</v>
+        <v>44.5</v>
       </c>
       <c r="H215">
         <v>172</v>
@@ -11741,13 +11741,13 @@
         <v>450</v>
       </c>
       <c r="F226">
-        <v>2</v>
+        <v>2.15</v>
       </c>
       <c r="G226">
-        <v>10.9</v>
+        <v>11.5</v>
       </c>
       <c r="H226">
-        <v>44.6</v>
+        <v>48</v>
       </c>
       <c r="I226" t="str">
         <v>Flaming Fox</v>
@@ -12124,7 +12124,7 @@
         <v>550</v>
       </c>
       <c r="H239">
-        <v>1465</v>
+        <v>1400</v>
       </c>
       <c r="I239" t="str">
         <v>Frost Dragon</v>
@@ -12205,13 +12205,13 @@
         <v>2300</v>
       </c>
       <c r="F242">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G242">
-        <v>56</v>
+        <v>59.5</v>
       </c>
       <c r="H242">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="I242" t="str">
         <v>Frost Unicorn</v>
@@ -12234,13 +12234,13 @@
         <v>2800</v>
       </c>
       <c r="F243">
-        <v>26.5</v>
+        <v>30</v>
       </c>
       <c r="G243">
-        <v>110</v>
+        <v>124</v>
       </c>
       <c r="H243">
-        <v>442</v>
+        <v>500</v>
       </c>
       <c r="I243" t="str">
         <v>Frostbite Bear</v>
@@ -12521,13 +12521,13 @@
         <v>230</v>
       </c>
       <c r="F253">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="G253">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="H253">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I253" t="str">
         <v>General Sheepdog</v>
@@ -12608,13 +12608,13 @@
         <v>300</v>
       </c>
       <c r="F256">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="G256">
-        <v>5.75</v>
+        <v>5.9</v>
       </c>
       <c r="H256">
-        <v>24</v>
+        <v>24.6</v>
       </c>
       <c r="I256" t="str">
         <v>Ghost Bunny</v>
@@ -12869,13 +12869,13 @@
         <v>30000</v>
       </c>
       <c r="F265">
-        <v>194</v>
+        <v>194.5</v>
       </c>
       <c r="G265">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="H265">
-        <v>2930</v>
+        <v>2960</v>
       </c>
       <c r="I265" t="str">
         <v>Giant Panda</v>
@@ -13107,7 +13107,7 @@
         <v>915</v>
       </c>
       <c r="H273">
-        <v>3100</v>
+        <v>2960</v>
       </c>
       <c r="I273" t="str">
         <v>Giraffe</v>
@@ -13159,13 +13159,13 @@
         <v>810</v>
       </c>
       <c r="F275">
-        <v>3.75</v>
+        <v>7.75</v>
       </c>
       <c r="G275">
-        <v>16.5</v>
+        <v>35</v>
       </c>
       <c r="H275">
-        <v>68</v>
+        <v>148</v>
       </c>
       <c r="I275" t="str">
         <v>Glacier Moth</v>
@@ -14116,13 +14116,13 @@
         <v>3930</v>
       </c>
       <c r="F308">
-        <v>23</v>
+        <v>23.25</v>
       </c>
       <c r="G308">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H308">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="I308" t="str">
         <v>Grim Dragon</v>
@@ -14319,13 +14319,13 @@
         <v>18500</v>
       </c>
       <c r="F315">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G315">
-        <v>417</v>
+        <v>427</v>
       </c>
       <c r="H315">
-        <v>1660</v>
+        <v>1725</v>
       </c>
       <c r="I315" t="str">
         <v>Haetae</v>
@@ -14464,13 +14464,13 @@
         <v>870</v>
       </c>
       <c r="F320">
-        <v>4</v>
+        <v>4.75</v>
       </c>
       <c r="G320">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H320">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I320" t="str">
         <v>Halloween White Ghost Dragon</v>
@@ -14580,13 +14580,13 @@
         <v>100</v>
       </c>
       <c r="F324">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="G324">
-        <v>1.95</v>
+        <v>1.9</v>
       </c>
       <c r="H324">
-        <v>8.25</v>
+        <v>8</v>
       </c>
       <c r="I324" t="str">
         <v>Hamster</v>
@@ -14783,7 +14783,7 @@
         <v>12000</v>
       </c>
       <c r="F331">
-        <v>66.5</v>
+        <v>66.75</v>
       </c>
       <c r="G331">
         <v>250</v>
@@ -14841,13 +14841,13 @@
         <v>1080</v>
       </c>
       <c r="F333">
-        <v>5.25</v>
+        <v>7.5</v>
       </c>
       <c r="G333">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="H333">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="I333" t="str">
         <v>Hero Gibbon</v>
@@ -14957,13 +14957,13 @@
         <v>960</v>
       </c>
       <c r="F337">
-        <v>4.25</v>
+        <v>6.25</v>
       </c>
       <c r="G337">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="H337">
-        <v>82</v>
+        <v>124</v>
       </c>
       <c r="I337" t="str">
         <v>Honey Badger</v>
@@ -15624,13 +15624,13 @@
         <v>1720</v>
       </c>
       <c r="F360">
-        <v>8.25</v>
+        <v>9.75</v>
       </c>
       <c r="G360">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="H360">
-        <v>146</v>
+        <v>172</v>
       </c>
       <c r="I360" t="str">
         <v>Irish Water Spaniel</v>
@@ -15711,13 +15711,13 @@
         <v>8220</v>
       </c>
       <c r="F363">
-        <v>57.5</v>
+        <v>58</v>
       </c>
       <c r="G363">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="H363">
-        <v>710</v>
+        <v>740</v>
       </c>
       <c r="I363" t="str">
         <v>Jekyll Hydra</v>
@@ -15740,13 +15740,13 @@
         <v>1940</v>
       </c>
       <c r="F364">
-        <v>9.75</v>
+        <v>10</v>
       </c>
       <c r="G364">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H364">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="I364" t="str">
         <v>Jellyfish</v>
@@ -15798,13 +15798,13 @@
         <v>980</v>
       </c>
       <c r="F366">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="G366">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H366">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="I366" t="str">
         <v>Jousting Horse</v>
@@ -16001,13 +16001,13 @@
         <v>200</v>
       </c>
       <c r="F373">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="G373">
-        <v>4.05</v>
+        <v>4.1</v>
       </c>
       <c r="H373">
-        <v>17.2</v>
+        <v>17.4</v>
       </c>
       <c r="I373" t="str">
         <v>Karate Gorilla</v>
@@ -16030,13 +16030,13 @@
         <v>280</v>
       </c>
       <c r="F374">
-        <v>0.95</v>
+        <v>3.5</v>
       </c>
       <c r="G374">
-        <v>6.65</v>
+        <v>17</v>
       </c>
       <c r="H374">
-        <v>26.9</v>
+        <v>70</v>
       </c>
       <c r="I374" t="str">
         <v>Kelp Captain</v>
@@ -16059,13 +16059,13 @@
         <v>45</v>
       </c>
       <c r="F375">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="G375">
-        <v>1.1</v>
+        <v>1.15</v>
       </c>
       <c r="H375">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="I375" t="str">
         <v>Kelp Crewmate</v>
@@ -16088,13 +16088,13 @@
         <v>65</v>
       </c>
       <c r="F376">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="G376">
-        <v>1.45</v>
+        <v>1.85</v>
       </c>
       <c r="H376">
-        <v>5.75</v>
+        <v>7.75</v>
       </c>
       <c r="I376" t="str">
         <v>Kelp Hunter</v>
@@ -16117,13 +16117,13 @@
         <v>50</v>
       </c>
       <c r="F377">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="G377">
-        <v>1.15</v>
+        <v>1.35</v>
       </c>
       <c r="H377">
-        <v>4.25</v>
+        <v>5.25</v>
       </c>
       <c r="I377" t="str">
         <v>Kelp Raider</v>
@@ -16204,13 +16204,13 @@
         <v>100</v>
       </c>
       <c r="F380">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="G380">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="H380">
-        <v>8.5</v>
+        <v>8.25</v>
       </c>
       <c r="I380" t="str">
         <v>King Penguin</v>
@@ -16610,13 +16610,13 @@
         <v>945</v>
       </c>
       <c r="F394">
-        <v>4.5</v>
+        <v>5.25</v>
       </c>
       <c r="G394">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H394">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="I394" t="str">
         <v>Lava Dragon</v>
@@ -16639,13 +16639,13 @@
         <v>320</v>
       </c>
       <c r="F395">
-        <v>1.05</v>
+        <v>0.97</v>
       </c>
       <c r="G395">
-        <v>7.25</v>
+        <v>6.79</v>
       </c>
       <c r="H395">
-        <v>30</v>
+        <v>27.5</v>
       </c>
       <c r="I395" t="str">
         <v>Lava Wolf</v>
@@ -17680,7 +17680,7 @@
         <v>88</v>
       </c>
       <c r="H431">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="I431" t="str">
         <v>Mermicorn</v>
@@ -17787,13 +17787,13 @@
         <v>850</v>
       </c>
       <c r="F435">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="G435">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H435">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="I435" t="str">
         <v>Midnight Dragon</v>
@@ -18013,13 +18013,13 @@
         <v>65</v>
       </c>
       <c r="F443">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="G443">
-        <v>1.9</v>
+        <v>1.85</v>
       </c>
       <c r="H443">
-        <v>8</v>
+        <v>7.75</v>
       </c>
       <c r="I443" t="str">
         <v>Momma Moose</v>
@@ -18103,10 +18103,10 @@
         <v>34.5</v>
       </c>
       <c r="G446">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H446">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="I446" t="str">
         <v>Monkey King</v>
@@ -18187,13 +18187,13 @@
         <v>3250</v>
       </c>
       <c r="F449">
-        <v>15.5</v>
+        <v>17</v>
       </c>
       <c r="G449">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H449">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="I449" t="str">
         <v>Moonbeam Peacock</v>
@@ -19323,7 +19323,7 @@
         <v>601</v>
       </c>
       <c r="H489">
-        <v>1980</v>
+        <v>1860</v>
       </c>
       <c r="I489" t="str">
         <v>Owl</v>
@@ -19404,13 +19404,13 @@
         <v>240</v>
       </c>
       <c r="F492">
-        <v>0.9</v>
+        <v>0.94</v>
       </c>
       <c r="G492">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
       <c r="H492">
-        <v>22.2</v>
+        <v>23</v>
       </c>
       <c r="I492" t="str">
         <v>Panda</v>
@@ -19526,7 +19526,7 @@
         <v>394</v>
       </c>
       <c r="H496">
-        <v>1050</v>
+        <v>1025</v>
       </c>
       <c r="I496" t="str">
         <v>Parrot</v>
@@ -19691,13 +19691,13 @@
         <v>540</v>
       </c>
       <c r="F502">
-        <v>2</v>
+        <v>1.65</v>
       </c>
       <c r="G502">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="H502">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="I502" t="str">
         <v>Peahen</v>
@@ -19778,10 +19778,10 @@
         <v>3000</v>
       </c>
       <c r="F505">
-        <v>26.5</v>
+        <v>26.75</v>
       </c>
       <c r="G505">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H505">
         <v>380</v>
@@ -19873,13 +19873,13 @@
         <v>1320</v>
       </c>
       <c r="F509">
-        <v>6.75</v>
+        <v>8</v>
       </c>
       <c r="G509">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H509">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="I509" t="str">
         <v>Phantom Dragon</v>
@@ -20134,13 +20134,13 @@
         <v>2640</v>
       </c>
       <c r="F518">
-        <v>14.75</v>
+        <v>15.75</v>
       </c>
       <c r="G518">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H518">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="I518" t="str">
         <v>Pirate Ghost Capuchin Monkey</v>
@@ -21172,13 +21172,13 @@
         <v>210</v>
       </c>
       <c r="F554">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="G554">
-        <v>4.15</v>
+        <v>4.1</v>
       </c>
       <c r="H554">
-        <v>17.6</v>
+        <v>17.4</v>
       </c>
       <c r="I554" t="str">
         <v>Ranger Beaver</v>
@@ -22642,13 +22642,13 @@
         <v>390</v>
       </c>
       <c r="F605">
-        <v>1.65</v>
+        <v>1.85</v>
       </c>
       <c r="G605">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
       <c r="H605">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="I605" t="str">
         <v>Scorching Kaijunior</v>
@@ -22909,7 +22909,7 @@
         <v>1343</v>
       </c>
       <c r="H614">
-        <v>3415</v>
+        <v>3320</v>
       </c>
       <c r="I614" t="str">
         <v>Shadow Dragon</v>
@@ -23367,13 +23367,13 @@
         <v>2000</v>
       </c>
       <c r="F630">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="G630">
-        <v>112</v>
+        <v>145</v>
       </c>
       <c r="H630">
-        <v>450</v>
+        <v>600</v>
       </c>
       <c r="I630" t="str">
         <v>Silverback Gorilla</v>
@@ -24382,13 +24382,13 @@
         <v>980</v>
       </c>
       <c r="F665">
-        <v>4.25</v>
+        <v>4.5</v>
       </c>
       <c r="G665">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H665">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I665" t="str">
         <v>Strawberry Penguin</v>
@@ -24417,7 +24417,7 @@
         <v>108</v>
       </c>
       <c r="H666">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="I666" t="str">
         <v>Strawberry Shortcake Bat Dragon</v>
@@ -24556,13 +24556,13 @@
         <v>1655</v>
       </c>
       <c r="F671">
-        <v>8</v>
+        <v>9.5</v>
       </c>
       <c r="G671">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="H671">
-        <v>142</v>
+        <v>170</v>
       </c>
       <c r="I671" t="str">
         <v>Sugar Axolotl</v>
@@ -25281,13 +25281,13 @@
         <v>1680</v>
       </c>
       <c r="F696">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G696">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="H696">
-        <v>158</v>
+        <v>200</v>
       </c>
       <c r="I696" t="str">
         <v>Tió De Nadal</v>
@@ -25310,13 +25310,13 @@
         <v>130</v>
       </c>
       <c r="F697">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="G697">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="H697">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="I697" t="str">
         <v>Toasty Red Panda</v>
@@ -25455,13 +25455,13 @@
         <v>265</v>
       </c>
       <c r="F702">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="G702">
-        <v>5.9</v>
+        <v>5.95</v>
       </c>
       <c r="H702">
-        <v>24.6</v>
+        <v>24.8</v>
       </c>
       <c r="I702" t="str">
         <v>Toy Monkey</v>
@@ -25629,13 +25629,13 @@
         <v>930</v>
       </c>
       <c r="F708">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="G708">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="H708">
-        <v>128</v>
+        <v>376</v>
       </c>
       <c r="I708" t="str">
         <v>Tri-Horned Treehopper</v>
@@ -25803,13 +25803,13 @@
         <v>9180</v>
       </c>
       <c r="F714">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G714">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H714">
-        <v>820</v>
+        <v>828</v>
       </c>
       <c r="I714" t="str">
         <v>Undead Jousting Horse</v>
@@ -25919,13 +25919,13 @@
         <v>1700</v>
       </c>
       <c r="F718">
-        <v>8.75</v>
+        <v>9</v>
       </c>
       <c r="G718">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H718">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="I718" t="str">
         <v>Vampire Dragon</v>
@@ -26006,13 +26006,13 @@
         <v>1440</v>
       </c>
       <c r="F721">
-        <v>7.75</v>
+        <v>7.5</v>
       </c>
       <c r="G721">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H721">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="I721" t="str">
         <v>Velocirooster</v>
@@ -26093,13 +26093,13 @@
         <v>330</v>
       </c>
       <c r="F724">
-        <v>0.98</v>
+        <v>1.05</v>
       </c>
       <c r="G724">
-        <v>6.86</v>
+        <v>7.25</v>
       </c>
       <c r="H724">
-        <v>27.8</v>
+        <v>30</v>
       </c>
       <c r="I724" t="str">
         <v>Violet Butterfly</v>
@@ -26415,10 +26415,10 @@
         <v>23</v>
       </c>
       <c r="G735">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H735">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="I735" t="str">
         <v>Werewolf</v>
@@ -26557,13 +26557,13 @@
         <v>210</v>
       </c>
       <c r="F740">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="G740">
-        <v>1.85</v>
+        <v>1.9</v>
       </c>
       <c r="H740">
-        <v>7.75</v>
+        <v>8</v>
       </c>
       <c r="I740" t="str">
         <v>Wildfire Hawk</v>
@@ -26615,13 +26615,13 @@
         <v>2520</v>
       </c>
       <c r="F742">
-        <v>12.25</v>
+        <v>13.75</v>
       </c>
       <c r="G742">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="H742">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="I742" t="str">
         <v>Winged Tiger</v>
@@ -26789,13 +26789,13 @@
         <v>520</v>
       </c>
       <c r="F748">
-        <v>1.97</v>
+        <v>2</v>
       </c>
       <c r="G748">
-        <v>10.75</v>
+        <v>11</v>
       </c>
       <c r="H748">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I748" t="str">
         <v>Wood Pigeon</v>
@@ -27012,13 +27012,13 @@
         <v>190</v>
       </c>
       <c r="F756">
-        <v>0.61</v>
+        <v>0.6</v>
       </c>
       <c r="G756">
-        <v>3.85</v>
+        <v>3.8</v>
       </c>
       <c r="H756">
-        <v>16.4</v>
+        <v>16.2</v>
       </c>
       <c r="I756" t="str">
         <v>Yeti</v>
@@ -27157,13 +27157,13 @@
         <v>1920</v>
       </c>
       <c r="F761">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="G761">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H761">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="I761" t="str">
         <v>Zombie Buffalo</v>
@@ -27215,13 +27215,13 @@
         <v>300</v>
       </c>
       <c r="F763">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="G763">
-        <v>6.05</v>
+        <v>6.15</v>
       </c>
       <c r="H763">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="I763" t="str">
         <v>Zombie Wolf</v>
@@ -27455,13 +27455,13 @@
         <v>/images/pets/Cake Friend.png</v>
       </c>
       <c r="F1001">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="G1001">
-        <v>6.15</v>
+        <v>6</v>
       </c>
       <c r="H1001">
-        <v>25.6</v>
+        <v>25</v>
       </c>
       <c r="I1001" t="str">
         <v>Cake Friend</v>
@@ -27569,21 +27569,55 @@
         <v>/images/pets/Wooly Rhino.png</v>
       </c>
       <c r="F1007">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="G1007">
-        <v>4.1</v>
+        <v>4.15</v>
       </c>
       <c r="H1007">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="I1007" t="str">
         <v>Wooly Rhino</v>
       </c>
     </row>
+    <row r="1008">
+      <c r="A1008" t="str">
+        <v>Chihuaha</v>
+      </c>
+      <c r="B1008" t="str">
+        <v>/images/pets/Chihuaha.png</v>
+      </c>
+      <c r="F1008">
+        <v>1.27</v>
+      </c>
+      <c r="G1008">
+        <v>7.25</v>
+      </c>
+      <c r="H1008">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="str">
+        <v>Tuxedo Cat</v>
+      </c>
+      <c r="B1009" t="str">
+        <v>/images/pets/Tuxedo Cat.png</v>
+      </c>
+      <c r="F1009">
+        <v>2</v>
+      </c>
+      <c r="G1009">
+        <v>11</v>
+      </c>
+      <c r="H1009">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1007"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1009"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -32893,7 +32927,7 @@
         <v>670</v>
       </c>
       <c r="F379">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="380" ht="19.5" customHeight="1">
@@ -32921,7 +32955,7 @@
         <v>450</v>
       </c>
       <c r="F381">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="382" ht="19.5" customHeight="1">
@@ -38772,7 +38806,7 @@
         <v>860</v>
       </c>
       <c r="F800">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="801" ht="19.5" customHeight="1">
@@ -38954,7 +38988,7 @@
         <v>940</v>
       </c>
       <c r="F813">
-        <v>151</v>
+        <v>190</v>
       </c>
     </row>
     <row r="814" ht="19.5" customHeight="1">
@@ -38982,7 +39016,7 @@
         <v>970</v>
       </c>
       <c r="F815">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="816" ht="19.5" customHeight="1">
@@ -40807,7 +40841,7 @@
         <v>/images/pets/Buzzing Honeypot Hat.png</v>
       </c>
       <c r="F1001">
-        <v>270</v>
+        <v>200</v>
       </c>
     </row>
     <row r="1002">
@@ -40818,7 +40852,7 @@
         <v>/images/pets/Hive Backpack.png</v>
       </c>
       <c r="F1002">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="1003">
@@ -40848,7 +40882,7 @@
         <v>/images/pets/Panda Cap.png</v>
       </c>
       <c r="F1005">
-        <v>1250</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="1006">
@@ -40859,7 +40893,7 @@
         <v>/images/pets/Queen Bee Slippers.png</v>
       </c>
       <c r="F1006">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row r="1007">
@@ -41324,7 +41358,7 @@
         <v>2500</v>
       </c>
       <c r="D33">
-        <v>198</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" ht="18.75" customHeight="1">
@@ -42957,7 +42991,7 @@
         <v>3445</v>
       </c>
       <c r="D96">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="97" ht="18.75" customHeight="1">

</xml_diff>